<commit_message>
tích hợp giao diện react, đóng gói docker
</commit_message>
<xml_diff>
--- a/QA.xlsx
+++ b/QA.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\RAG-TC-DL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A786112-0FCE-4F46-9D32-7BABEA4B10DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECAF9504-C790-4F86-A1ED-8394A4D0C28F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="112">
   <si>
     <t>1. Phạm vi đo lường của van an toàn trong QTKĐ 1.061 là bao nhiêu?</t>
   </si>
@@ -349,6 +349,18 @@
   </si>
   <si>
     <t>AKKĐ là viết tắt của "Áp kế chuẩn, chân không kế chuẩn". Đây thường được sử dụng trong các quy trình kiểm định đo lường để xác nhận chính xác của thiết bị đo áp suất. AKKĐ có phạm vi đo từ -1 bar đến 5000 bar và cấp chính xác đến 0,02%.</t>
+  </si>
+  <si>
+    <t>Áp suất chuẩn trong chế độ đo áp suất tương đối tại điểm kiểm tra thứ i ứng với điểm mốc cơ sở áp suất của áp kế píttông chuẩn được tính theo công thức</t>
+  </si>
+  <si>
+    <t>Áp suất chuẩn trong chế độ đo áp suất tương đối tại điểm kiểm tra thứ i i ứng với điểm mốc cơ sở áp suất của áp kế pít tông chuẩn có thể được tính theo công thức: P i = P 0 + Δ P i P i ​ =P 0 ​ +ΔP i ​ Trong đó: P i P i ​ là áp suất chuẩn tại điểm kiểm tra thứ i i. P 0 P 0 ​ là áp suất mốc cơ sở của pít tông chuẩn. Δ P i ΔP i ​ là sự thay đổi áp suất do môi trường truyền áp suất và điều kiện đo tại điểm kiểm tra thứ i i. Cụ thể, nếu bạn đang sử dụng hệ thống đo áp suất tương đối, thì Δ P i ΔP i ​ thường bao gồm các yếu tố như độ nhớt của môi trường truyền áp suất, tốc độ quay tự do của pít tông, và các thay đổi khác do điều kiện đo tại điểm kiểm tra thứ i i. Ví dụ cụ thể có thể phụ thuộc vào quy trình kiểm định cụ thể mà bạn đang sử dụng. Nếu cần thêm thông tin chi tiết về từng yếu tố này, xin vui lòng cung cấp thêm thông tin về hệ thống đo cụ thể của bạn.</t>
+  </si>
+  <si>
+    <t>diện tích hiệu dụng của píttông của AKKĐ tại điểm kiểm tra thứ i được tính từ công thức nào</t>
+  </si>
+  <si>
+    <t>Xác định hệ số tuyến tính R như thế nào</t>
   </si>
 </sst>
 </file>
@@ -400,7 +412,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -414,6 +426,12 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -695,7 +713,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:C60"/>
+  <dimension ref="B1:C66"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="8.7265625" style="1"/>
@@ -749,7 +767,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="2:3" ht="201.5" x14ac:dyDescent="0.4">
+    <row r="7" spans="2:3" ht="170.5" x14ac:dyDescent="0.4">
       <c r="B7" s="2" t="s">
         <v>5</v>
       </c>
@@ -771,7 +789,7 @@
       </c>
       <c r="C9" s="5"/>
     </row>
-    <row r="10" spans="2:3" ht="46.5" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:3" ht="31" x14ac:dyDescent="0.4">
       <c r="B10" s="2" t="s">
         <v>9</v>
       </c>
@@ -779,7 +797,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="11" spans="2:3" ht="139.5" x14ac:dyDescent="0.4">
+    <row r="11" spans="2:3" ht="124" x14ac:dyDescent="0.4">
       <c r="B11" s="2" t="s">
         <v>10</v>
       </c>
@@ -833,7 +851,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="18" spans="2:3" ht="186" x14ac:dyDescent="0.4">
+    <row r="18" spans="2:3" ht="170.5" x14ac:dyDescent="0.4">
       <c r="B18" s="2" t="s">
         <v>17</v>
       </c>
@@ -841,7 +859,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="19" spans="2:3" ht="108.5" x14ac:dyDescent="0.4">
+    <row r="19" spans="2:3" ht="93" x14ac:dyDescent="0.4">
       <c r="B19" s="2" t="s">
         <v>18</v>
       </c>
@@ -909,7 +927,7 @@
       </c>
       <c r="C27" s="5"/>
     </row>
-    <row r="28" spans="2:3" ht="46.5" x14ac:dyDescent="0.4">
+    <row r="28" spans="2:3" ht="31" x14ac:dyDescent="0.4">
       <c r="B28" s="2" t="s">
         <v>27</v>
       </c>
@@ -987,7 +1005,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="38" spans="2:3" ht="108.5" x14ac:dyDescent="0.4">
+    <row r="38" spans="2:3" ht="93" x14ac:dyDescent="0.4">
       <c r="B38" s="2" t="s">
         <v>37</v>
       </c>
@@ -1017,7 +1035,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="42" spans="2:3" ht="77.5" x14ac:dyDescent="0.4">
+    <row r="42" spans="2:3" ht="62" x14ac:dyDescent="0.4">
       <c r="B42" s="2" t="s">
         <v>41</v>
       </c>
@@ -1047,7 +1065,7 @@
       </c>
       <c r="C45" s="5"/>
     </row>
-    <row r="46" spans="2:3" ht="46.5" x14ac:dyDescent="0.4">
+    <row r="46" spans="2:3" ht="31" x14ac:dyDescent="0.4">
       <c r="B46" s="2" t="s">
         <v>45</v>
       </c>
@@ -1055,7 +1073,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="47" spans="2:3" ht="155" x14ac:dyDescent="0.4">
+    <row r="47" spans="2:3" ht="139.5" x14ac:dyDescent="0.4">
       <c r="B47" s="2" t="s">
         <v>46</v>
       </c>
@@ -1063,7 +1081,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="48" spans="2:3" ht="77.5" x14ac:dyDescent="0.4">
+    <row r="48" spans="2:3" ht="62" x14ac:dyDescent="0.4">
       <c r="B48" s="2" t="s">
         <v>47</v>
       </c>
@@ -1071,7 +1089,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="49" spans="2:3" ht="108.5" x14ac:dyDescent="0.4">
+    <row r="49" spans="2:3" ht="93" x14ac:dyDescent="0.4">
       <c r="B49" s="2" t="s">
         <v>48</v>
       </c>
@@ -1087,7 +1105,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="51" spans="2:3" ht="62" x14ac:dyDescent="0.4">
+    <row r="51" spans="2:3" ht="46.5" x14ac:dyDescent="0.4">
       <c r="B51" s="2" t="s">
         <v>50</v>
       </c>
@@ -1095,7 +1113,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="52" spans="2:3" ht="77.5" x14ac:dyDescent="0.4">
+    <row r="52" spans="2:3" ht="62" x14ac:dyDescent="0.4">
       <c r="B52" s="2" t="s">
         <v>51</v>
       </c>
@@ -1125,7 +1143,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="56" spans="2:3" ht="31" x14ac:dyDescent="0.4">
+    <row r="56" spans="2:3" x14ac:dyDescent="0.4">
       <c r="B56" s="2" t="s">
         <v>55</v>
       </c>
@@ -1147,7 +1165,7 @@
       </c>
       <c r="C58" s="5"/>
     </row>
-    <row r="59" spans="2:3" ht="155" x14ac:dyDescent="0.4">
+    <row r="59" spans="2:3" ht="139.5" x14ac:dyDescent="0.4">
       <c r="B59" s="2" t="s">
         <v>58</v>
       </c>
@@ -1161,6 +1179,24 @@
       </c>
       <c r="C60" s="5" t="s">
         <v>107</v>
+      </c>
+    </row>
+    <row r="64" spans="2:3" ht="162" x14ac:dyDescent="0.4">
+      <c r="B64" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="C64" s="4" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="65" spans="2:2" ht="36" x14ac:dyDescent="0.4">
+      <c r="B65" s="7" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="66" spans="2:2" x14ac:dyDescent="0.4">
+      <c r="B66" s="6" t="s">
+        <v>111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>